<commit_message>
Reporte Integrado BORA-COMPRAR-TGN: 2026-02-23
</commit_message>
<xml_diff>
--- a/data/2026-02/flujo_licitaciones_2026-02-23.xlsx
+++ b/data/2026-02/flujo_licitaciones_2026-02-23.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ Adjudicados con CUIT" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔗 Flujo Cruzado" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⏳ Licitaciones Abiertas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚠️ Alertas Riesgo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -539,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,6 +624,26 @@
           <t>alerta</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>indicadores_riesgo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>score_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>indice_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>nivel_riesgo_licit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -632,12 +653,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MINISTERIO PÚBLICO DE LA DEFENSA -</t>
+          <t>MINISTERIO PÚBLICO DE LA DEFENSA - DEFENSORÍA GENERAL DE LA NACIÓN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DEFENSORÍA GENERAL DE LA NACIÓN</t>
+          <t>Licitación Pública 49/2025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -675,6 +696,22 @@
           <t>📋 SOLO BORA</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -684,12 +721,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MINISTERIO PÚBLICO DE LA DEFENSA -</t>
+          <t>MINISTERIO PÚBLICO DE LA DEFENSA - DEFENSORÍA GENERAL DE LA NACIÓN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DEFENSORÍA GENERAL DE LA NACIÓN</t>
+          <t>Licitación Pública 59/2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -727,6 +764,22 @@
           <t>📋 SOLO BORA</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -779,6 +832,22 @@
           <t>📋 SOLO BORA</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -788,12 +857,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO -</t>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CENTRAL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DIRECCIÓN REGIONAL ADUANERA CENTRAL</t>
+          <t>Contratación Directa 01/26</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -837,6 +906,22 @@
       <c r="P5" t="inlineStr">
         <is>
           <t>📋 SOLO BORA</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S5" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
     </row>
@@ -891,6 +976,22 @@
           <t>📋 SOLO BORA</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -943,6 +1044,22 @@
           <t>📋 SOLO BORA</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -997,6 +1114,22 @@
       <c r="P8" t="inlineStr">
         <is>
           <t>📋 SOLO BORA</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Bajo</t>
         </is>
       </c>
     </row>
@@ -1069,22 +1202,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>487-0101-LPU25</t>
+          <t>84/11-2048-LPR25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Servicio para la recepción, elaboración y distribución de alimentos.</t>
+          <t>CONTRATAR UN SERVICIO PARA LA PERFORACIÓN DE POZO DE AGUA.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1094,7 +1227,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>487 - División Compras y Suministros - Superintendencia de Bienestar de la Policia Federal Argentina</t>
+          <t>84/11 - Liceo Militar General San Martin</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1116,22 +1249,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>38/15-0012-LPU26</t>
+          <t>84/11-2119-LPR25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Servicio de locación, mantenimiento y gestión de impresiones digitales (Impresión y Fotocopiado)</t>
+          <t>CONTRATAR UN SERVICIO DE MANTENIMIENTO Y LIMPIEZA DE LA RED CLOACAL Y CÁMARAS SEPTICAS.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1141,7 +1274,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>38/15 JEFATURA DE OBTENCION DE LA ARMADA</t>
+          <t>84/11 - Liceo Militar General San Martin</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1163,12 +1296,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>40/47-0629-LPR25</t>
+          <t>84/71-0038-LPR26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Servicio de Fotocopiadora para la ESCUELA DE AVAICION MILITAR</t>
+          <t>CONTRATACIÓN DEL SERVICIO DE HOSTING WEB ANUAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1178,7 +1311,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1188,7 +1321,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Departamento Contrataciones Córdoba - UOC 40/47</t>
+          <t>84/71 - Liceo Militar General Roca</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1210,22 +1343,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>38/18-0063-LPR26</t>
+          <t>40/16-0062-CDI26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PROVISIÓN DE CARTAS ELECTRÓNICAS PERTENECIENTES AL BUQUE ESCUELA FRAGATA A.R.A. "LIBERTAD".</t>
+          <t>ADQUISICION DE SERVICIO DE RESIDUOS PATOLOGICOS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1235,7 +1368,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>38/18 - Division Contrataciones - Comando de Transportes Navales</t>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1257,22 +1390,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>38/18-0057-LPR26</t>
+          <t>40/16-0036-CDI26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MANTENIMIENTO DE CAMARAS Y COMPRESORES DE FRIGORIFICA PARA EL BUQUE ESCUELA A.R.A. "LIBERTAD"</t>
+          <t>ADQUISICION DE MATERIALES ELECTRICOS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1282,7 +1415,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>38/18 - Division Contrataciones - Comando de Transportes Navales</t>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1304,22 +1437,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>37/20-0939-CDI25</t>
+          <t>40/16-0017-LPR26</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ALQUILER DE DISPENSERS DE AGUA FRIO/CALOR</t>
+          <t>ADQUISICIÓN DE INSUMOS CÁRNICOS PAR ELABORACIÓN DE ALIMENTOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1329,7 +1462,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>37/020 - Escuadrón 4 "Concordia"</t>
+          <t>40/016 - AREA MATERIAL QUILMES</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1351,12 +1484,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>40/51-0023-LPR26</t>
+          <t>74/45-0023-LPR26</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Adquisición de Medicamentos Analgésicos, Antiinflamatorios, Psicotrópicos, Y Otros Para El HACBA.</t>
+          <t>ADQUISICION DE HERRAMIENTAS ELECTRICAS MENORES PARA EL PN ISLAS DE SANTA FE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1366,7 +1499,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 08:00 Hrs.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1376,7 +1509,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Departamento Contrataciones Córdoba - UOC 40/51</t>
+          <t>74/45 - Parque Nacional Islas de Santa Fe</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1398,22 +1531,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>84/19-0091-LPR26</t>
+          <t>39-0004-LPU26</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE MATERIALES DE FERRETERIA Y ELECTRICIDAD PARA EL CDO BR M VIII Y UU - 2DO TRIM 2026</t>
+          <t>ADQUISICIÓN E INSTALACIÓN DE CUATRO (4) COMPRESORES DE AIRE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>23/02/2026 10:00 Hrs.</t>
+          <t>24/02/2026 09:00 Hrs.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1423,7 +1556,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>84/19 - Comando Brigada de Montaña VIII</t>
+          <t>39 - Dirección General de Administración- PNA</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1445,22 +1578,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>40/23-0984-CDI25</t>
+          <t>38/3-1320-LPR25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SERVICIO DE FUMIGACION</t>
+          <t>ADQUISICION DE REPUESTOS PARA MOTOR FUERA DE BORDA (BNPB)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>23/02/2026 10:30 Hrs.</t>
+          <t>24/02/2026 09:00 Hrs.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1470,7 +1603,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>40/023 - DIVISIÓN CONTRATACIONES MORENO</t>
+          <t>38/03 - UOC de la Intendencia Naval Puerto Belgrano - Armada Argentina</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1492,12 +1625,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>84/71-0006-LPR26</t>
+          <t>38/3-1638-LPR25</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SERVICIO DE TRANSPORTE DEL PERSONAL DEL INSTITUTO</t>
+          <t>ADQUISICION DE MATERIALES ELECTRICOS PARA LAS SUBESTACIONES (BNPB)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1507,7 +1640,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>23/02/2026 12:00 Hrs.</t>
+          <t>24/02/2026 09:00 Hrs.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1517,7 +1650,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>84/71 - Liceo Militar General Roca</t>
+          <t>38/03 - UOC de la Intendencia Naval Puerto Belgrano - Armada Argentina</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1622,6 +1755,198 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>Comprar.gob.ar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fecha</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>organismo_contratante</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>tipo_proceso_bora</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>link_bora</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>proveedor_adjudicado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>cuit_proveedor</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>monto_adjudicado_bora</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>en_comprar</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>procesos_comprar</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>unidad_comprar</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>nro_proceso_comprar</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>cobro_en_tgn</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>beneficiario_tgn</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>monto_cobrado_tgn</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>etapa</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>alerta</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>indicadores_riesgo</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>score_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>indice_riesgo_licit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>nivel_riesgo_licit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENCIA DE RECAUDACIÓN Y CONTROL ADUANERO - DIRECCIÓN REGIONAL ADUANERA CENTRAL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Contratación Directa 01/26</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.boletinoficial.gob.ar/detalleAviso/tercera/2407959/20260223</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ELEVAR SRL</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>$1.164.000,00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>❌ NO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>⚠️ SIN CUIT EXTRAÍDO</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>📋 SOLO BORA</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>🔴 Contratación Directa | 🟡 Adjudicación mismo día de publicación</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="S2" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Medio</t>
         </is>
       </c>
     </row>

</xml_diff>